<commit_message>
Add: SI, LACMA 추가
</commit_message>
<xml_diff>
--- a/data/VA_hyungbae.xlsx
+++ b/data/VA_hyungbae.xlsx
@@ -5589,7 +5589,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>silk; gold thread</t>
+          <t>ink; paper</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -5599,7 +5599,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Height: 27.6cm; Width: 26.6cm</t>
+          <t>Width: 9cm; Length: 14cm</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">

</xml_diff>